<commit_message>
Corregimos sección Ambiente para que no corte el ciclo si el df tiene datos faltantes.
</commit_message>
<xml_diff>
--- a/Analisis_Anios_Nino_Localidades.xlsx
+++ b/Analisis_Anios_Nino_Localidades.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://intaarg-my.sharepoint.com/personal/lewczuk_nuria_inta_gob_ar/Documents/shiny_app/app_EMCBalcarce/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_3EB8ADA82F144CBE849A676EBA857A1C390CE135" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{424FC6C5-1E0B-4376-BE54-7B840BBCCAAC}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_3EB8ADA82F144CBE849A676EBA857A1C390CE135" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E867DA8-6D2B-4F22-A0A5-E73C84D973AC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20610" yWindow="4575" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Balcarce" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,20 @@
     <sheet name="BenitoJuarez" sheetId="6" r:id="rId6"/>
     <sheet name="Notas_metodologicas" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -7985,7 +7998,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:109" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:109" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>1972</v>
       </c>

</xml_diff>